<commit_message>
fixed delayed dashboard, synced between devices, tombol detail tersimpan improvement, excel export overwrite templates fixed, dynamic column insertion
</commit_message>
<xml_diff>
--- a/templates/DAILY REPORT_Tamplates.xlsx
+++ b/templates/DAILY REPORT_Tamplates.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_YX0BMK4C\Documents\RIKO\Apps\Act\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA5FE40-7A18-4569-A5B3-CB59A0156F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F19F75C-B88B-429D-A1BD-418A53019B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AD41AF38-EF9C-46FA-9496-695CF84B5875}"/>
+    <workbookView xWindow="0" yWindow="1103" windowWidth="21600" windowHeight="11332" xr2:uid="{AD41AF38-EF9C-46FA-9496-695CF84B5875}"/>
   </bookViews>
   <sheets>
     <sheet name="2026-9" sheetId="23" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'2026-9'!$B$1:$I$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'2026-9'!$B$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <r>
       <t xml:space="preserve">AKTIVITAS-AKTIVITAS IT / </t>
@@ -201,9 +201,6 @@
     </r>
   </si>
   <si>
-    <t>Finish</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Tgl. / </t>
     </r>
@@ -327,22 +324,7 @@
     <t>Riko Hermansyah</t>
   </si>
   <si>
-    <t>Bintan / IT Server</t>
-  </si>
-  <si>
-    <t>HW &amp; SW</t>
-  </si>
-  <si>
-    <t>120 Minutes</t>
-  </si>
-  <si>
-    <t>01/09/2026</t>
-  </si>
-  <si>
     <t>2026-09</t>
-  </si>
-  <si>
-    <t>EXAMPLE</t>
   </si>
 </sst>
 </file>
@@ -2202,7 +2184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -2230,21 +2212,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -2353,36 +2320,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -2660,7 +2597,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2707,56 +2644,56 @@
     <xf numFmtId="164" fontId="259" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="264" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="264" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="264" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="264" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="264" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="253" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="253" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="264" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="264" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="264" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="264" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="264" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="4" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="3" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="265" fillId="0" borderId="1" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2765,41 +2702,23 @@
     <xf numFmtId="0" fontId="265" fillId="0" borderId="1" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="17" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="14" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="16" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="13" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="5" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="4" xfId="135" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="14" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="3" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="3" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="15" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="251" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="251" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="251" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="251" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="251" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="239" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="250">
@@ -3496,7 +3415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F4C6F7-9C82-45E7-8B2F-59657E08894B}">
-  <dimension ref="B1:N353"/>
+  <dimension ref="B1:N351"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.1328125" customWidth="1"/>
@@ -4173,16 +4092,16 @@
       <c r="I5" s="26"/>
     </row>
     <row r="6" spans="2:14" ht="22.9" x14ac:dyDescent="0.65">
-      <c r="B6" s="51" t="s">
+      <c r="B6" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="53"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="49"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" s="25"/>
@@ -4201,7 +4120,7 @@
         <v>3</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="26"/>
@@ -4237,113 +4156,77 @@
       </c>
     </row>
     <row r="11" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="50" t="s">
+      <c r="B11" s="45"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="46"/>
+      <c r="M11" s="40"/>
+      <c r="N11" s="40"/>
+    </row>
+    <row r="12" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="37"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="24"/>
+    </row>
+    <row r="13" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="25"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="26"/>
+    </row>
+    <row r="14" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="27"/>
+      <c r="C14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="M11" s="40"/>
-    </row>
-    <row r="12" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="50" t="s">
+      <c r="D14" s="18"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="M12" s="40"/>
-    </row>
-    <row r="13" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="45"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="46"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="40"/>
-    </row>
-    <row r="14" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="37"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="24"/>
-    </row>
-    <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="25"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="21"/>
+      <c r="G14" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="20"/>
+      <c r="I14" s="26"/>
+    </row>
+    <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="27"/>
+      <c r="C15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="18"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="20"/>
       <c r="I15" s="26"/>
     </row>
     <row r="16" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B16" s="27"/>
-      <c r="C16" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="C16" s="12"/>
       <c r="D16" s="18"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>14</v>
-      </c>
+      <c r="F16" s="12"/>
       <c r="H16" s="20"/>
       <c r="I16" s="26"/>
     </row>
     <row r="17" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B17" s="27"/>
-      <c r="C17" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="C17" s="12"/>
       <c r="D17" s="18"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="12" t="s">
-        <v>16</v>
-      </c>
+      <c r="F17" s="12"/>
       <c r="H17" s="20"/>
       <c r="I17" s="26"/>
     </row>
@@ -4358,57 +4241,57 @@
     </row>
     <row r="19" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B19" s="27"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="18"/>
+      <c r="C19" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="19"/>
       <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+      <c r="F19" s="14" t="s">
+        <v>20</v>
+      </c>
       <c r="H19" s="20"/>
       <c r="I19" s="26"/>
     </row>
     <row r="20" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B20" s="27"/>
-      <c r="C20" s="12"/>
+      <c r="C20" s="12" t="s">
+        <v>16</v>
+      </c>
       <c r="D20" s="18"/>
       <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
+      <c r="F20" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="H20" s="20"/>
       <c r="I20" s="26"/>
     </row>
-    <row r="21" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="27"/>
-      <c r="C21" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="19"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="20"/>
-      <c r="I21" s="26"/>
-    </row>
-    <row r="22" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="27"/>
-      <c r="C22" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12" t="s">
-        <v>18</v>
-      </c>
+    <row r="21" spans="2:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="28"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="32"/>
+    </row>
+    <row r="22" spans="2:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C22"/>
+      <c r="D22" s="15"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
       <c r="H22" s="20"/>
-      <c r="I22" s="26"/>
-    </row>
-    <row r="23" spans="2:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="32"/>
+      <c r="I22" s="15"/>
+    </row>
+    <row r="23" spans="2:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C23"/>
+      <c r="D23" s="15"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="15"/>
     </row>
     <row r="24" spans="2:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C24"/>
@@ -4536,23 +4419,11 @@
       <c r="H37" s="20"/>
       <c r="I37" s="15"/>
     </row>
-    <row r="38" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C38"/>
-      <c r="D38" s="15"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
+    <row r="38" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H38" s="20"/>
-      <c r="I38" s="15"/>
-    </row>
-    <row r="39" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C39"/>
-      <c r="D39" s="15"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
+    </row>
+    <row r="39" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H39" s="20"/>
-      <c r="I39" s="15"/>
     </row>
     <row r="40" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H40" s="20"/>
@@ -4576,21 +4447,33 @@
       <c r="H46" s="20"/>
     </row>
     <row r="47" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="H47" s="20"/>
+      <c r="H47" s="20" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="48" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H48" s="20"/>
     </row>
     <row r="49" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="H49" s="20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="50" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H49" s="20"/>
+    </row>
+    <row r="50" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C50"/>
+      <c r="D50" s="15"/>
+      <c r="E50"/>
+      <c r="F50"/>
+      <c r="G50"/>
       <c r="H50" s="20"/>
-    </row>
-    <row r="51" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I50" s="15"/>
+    </row>
+    <row r="51" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C51"/>
+      <c r="D51" s="15"/>
+      <c r="E51"/>
+      <c r="F51"/>
+      <c r="G51"/>
       <c r="H51" s="20"/>
+      <c r="I51" s="15"/>
     </row>
     <row r="52" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C52"/>
@@ -5228,7 +5111,7 @@
       <c r="E122"/>
       <c r="F122"/>
       <c r="G122"/>
-      <c r="H122" s="20"/>
+      <c r="H122"/>
       <c r="I122" s="15"/>
     </row>
     <row r="123" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -5237,7 +5120,7 @@
       <c r="E123"/>
       <c r="F123"/>
       <c r="G123"/>
-      <c r="H123" s="20"/>
+      <c r="H123"/>
       <c r="I123" s="15"/>
     </row>
     <row r="124" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -5870,26 +5753,26 @@
       <c r="H193"/>
       <c r="I193" s="15"/>
     </row>
-    <row r="194" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C194"/>
-      <c r="D194" s="15"/>
-      <c r="E194"/>
-      <c r="F194"/>
-      <c r="G194"/>
-      <c r="H194"/>
-      <c r="I194" s="15"/>
-    </row>
-    <row r="195" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C195"/>
-      <c r="D195" s="15"/>
-      <c r="E195"/>
-      <c r="F195"/>
-      <c r="G195"/>
-      <c r="H195"/>
-      <c r="I195" s="15"/>
-    </row>
-    <row r="196" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="197" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="194" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="195" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="196" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C196"/>
+      <c r="D196" s="15"/>
+      <c r="E196"/>
+      <c r="F196"/>
+      <c r="G196"/>
+      <c r="H196"/>
+      <c r="I196" s="15"/>
+    </row>
+    <row r="197" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C197"/>
+      <c r="D197" s="15"/>
+      <c r="E197"/>
+      <c r="F197"/>
+      <c r="G197"/>
+      <c r="H197"/>
+      <c r="I197" s="15"/>
+    </row>
     <row r="198" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C198"/>
       <c r="D198" s="15"/>
@@ -6016,24 +5899,8 @@
       <c r="H211"/>
       <c r="I211" s="15"/>
     </row>
-    <row r="212" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C212"/>
-      <c r="D212" s="15"/>
-      <c r="E212"/>
-      <c r="F212"/>
-      <c r="G212"/>
-      <c r="H212"/>
-      <c r="I212" s="15"/>
-    </row>
-    <row r="213" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C213"/>
-      <c r="D213" s="15"/>
-      <c r="E213"/>
-      <c r="F213"/>
-      <c r="G213"/>
-      <c r="H213"/>
-      <c r="I213" s="15"/>
-    </row>
+    <row r="212" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="213" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="214" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="215" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="216" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -6048,8 +5915,24 @@
     <row r="225" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="226" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="227" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="228" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="229" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="228" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C228"/>
+      <c r="D228" s="15"/>
+      <c r="E228"/>
+      <c r="F228"/>
+      <c r="G228"/>
+      <c r="H228"/>
+      <c r="I228" s="15"/>
+    </row>
+    <row r="229" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C229"/>
+      <c r="D229" s="15"/>
+      <c r="E229"/>
+      <c r="F229"/>
+      <c r="G229"/>
+      <c r="H229"/>
+      <c r="I229" s="15"/>
+    </row>
     <row r="230" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C230"/>
       <c r="D230" s="15"/>
@@ -6716,7 +6599,7 @@
       <c r="H303"/>
       <c r="I303" s="15"/>
     </row>
-    <row r="304" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="3:9" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C304"/>
       <c r="D304" s="15"/>
       <c r="E304"/>
@@ -6725,7 +6608,7 @@
       <c r="H304"/>
       <c r="I304" s="15"/>
     </row>
-    <row r="305" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="3:9" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C305"/>
       <c r="D305" s="15"/>
       <c r="E305"/>
@@ -7130,7 +7013,7 @@
       <c r="H349"/>
       <c r="I349" s="15"/>
     </row>
-    <row r="350" spans="3:9" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C350"/>
       <c r="D350" s="15"/>
       <c r="E350"/>
@@ -7139,7 +7022,7 @@
       <c r="H350"/>
       <c r="I350" s="15"/>
     </row>
-    <row r="351" spans="3:9" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C351"/>
       <c r="D351" s="15"/>
       <c r="E351"/>
@@ -7147,24 +7030,6 @@
       <c r="G351"/>
       <c r="H351"/>
       <c r="I351" s="15"/>
-    </row>
-    <row r="352" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C352"/>
-      <c r="D352" s="15"/>
-      <c r="E352"/>
-      <c r="F352"/>
-      <c r="G352"/>
-      <c r="H352"/>
-      <c r="I352" s="15"/>
-    </row>
-    <row r="353" spans="3:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C353"/>
-      <c r="D353" s="15"/>
-      <c r="E353"/>
-      <c r="F353"/>
-      <c r="G353"/>
-      <c r="H353"/>
-      <c r="I353" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
change excel template to october
</commit_message>
<xml_diff>
--- a/templates/DAILY REPORT_Tamplates.xlsx
+++ b/templates/DAILY REPORT_Tamplates.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_YX0BMK4C\Documents\RIKO\Apps\Act\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F19F75C-B88B-429D-A1BD-418A53019B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5D517A-FC49-459E-8821-35C16AA9B628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1103" windowWidth="21600" windowHeight="11332" xr2:uid="{AD41AF38-EF9C-46FA-9496-695CF84B5875}"/>
+    <workbookView xWindow="-28898" yWindow="-2820" windowWidth="28996" windowHeight="15675" xr2:uid="{AD41AF38-EF9C-46FA-9496-695CF84B5875}"/>
   </bookViews>
   <sheets>
-    <sheet name="2026-9" sheetId="23" r:id="rId1"/>
+    <sheet name="2026-10" sheetId="23" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'2026-9'!$B$1:$I$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'2026-10'!$B$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -324,7 +324,7 @@
     <t>Riko Hermansyah</t>
   </si>
   <si>
-    <t>2026-09</t>
+    <t>2026-10</t>
   </si>
 </sst>
 </file>

</xml_diff>